<commit_message>
auto: add 01-Projects (2), modify 01-Projects (6), modify 02-Knowledge (2)
</commit_message>
<xml_diff>
--- a/01-Projects/family-investment/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-investment/credit-card-management/信用卡主控表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11565"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11565" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="1-卡片信息" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="344">
   <si>
     <t>信用卡卡片总览 — 韩伟</t>
   </si>
@@ -209,9 +209,6 @@
   </si>
   <si>
     <t>普通白金卡</t>
-  </si>
-  <si>
-    <t>【已办理】年费980→25W积分抵；权益：299酒店/代驾20km/贵宾厅4次</t>
   </si>
   <si>
     <t>交通银行</t>
@@ -995,15 +992,6 @@
     <t>待记录</t>
   </si>
   <si>
-    <t>提额</t>
-  </si>
-  <si>
-    <t>APP人工提额度，授权了个税记录</t>
-  </si>
-  <si>
-    <t>待结果</t>
-  </si>
-  <si>
     <t>申请12W</t>
   </si>
   <si>
@@ -1020,10 +1008,6 @@
   </si>
   <si>
     <t>没有申请按钮，需要分期？</t>
-  </si>
-  <si>
-    <t>19日</t>
-    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>18日</t>
@@ -1059,6 +1043,108 @@
   </si>
   <si>
     <t>15日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>笔</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>兑换里程</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>银行APP直接搜索年费查询
+6月-9月可兑换</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>日</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>16日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>【已办理】年费980→25W积分抵；权益：299酒店/代驾20km/贵宾厅4次</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">普通白金卡
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>积分可兑换南航</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>积分可兑换里程</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">值得办理 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 可办理燕的那个
+积分兑换里程</t>
+    </r>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -1216,7 +1302,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1293,6 +1379,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -1405,7 +1503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1541,6 +1639,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1568,6 +1672,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1982,15 +2101,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2184,7 +2303,7 @@
         <v>50000</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="H9" s="28"/>
     </row>
@@ -2234,7 +2353,7 @@
         <v>26000</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="H11" s="28"/>
     </row>
@@ -2407,12 +2526,12 @@
       <c r="H18" s="28"/>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="56"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="58"/>
       <c r="E19" s="3">
         <v>919000</v>
       </c>
@@ -2423,26 +2542,26 @@
       <c r="H19" s="28"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="52"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="51" t="s">
+      <c r="A24" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="54"/>
+      <c r="G24" s="54"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="40" t="s">
@@ -2470,37 +2589,41 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1">
+    <row r="26" spans="1:8" ht="32.25" customHeight="1">
       <c r="A26" s="37">
         <v>1</v>
       </c>
       <c r="B26" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="37" t="s">
-        <v>59</v>
+      <c r="C26" s="52" t="s">
+        <v>341</v>
       </c>
       <c r="D26" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="28" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="16.5" customHeight="1">
+      <c r="E26" s="41">
+        <v>11000</v>
+      </c>
+      <c r="F26" s="41">
+        <v>11000</v>
+      </c>
+      <c r="G26" s="52" t="s">
+        <v>338</v>
+      </c>
+      <c r="H26" s="69" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="31.5" customHeight="1">
       <c r="A27" s="37">
         <v>2</v>
       </c>
       <c r="B27" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="37" t="s">
         <v>61</v>
-      </c>
-      <c r="C27" s="37" t="s">
-        <v>62</v>
       </c>
       <c r="D27" s="37" t="s">
         <v>11</v>
@@ -2510,11 +2633,11 @@
       <c r="G27" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H27" s="28" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="16.5" customHeight="1">
+      <c r="H27" s="69" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="36.75" customHeight="1">
       <c r="A28" s="37">
         <v>3</v>
       </c>
@@ -2522,7 +2645,7 @@
         <v>42</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D28" s="37" t="s">
         <v>11</v>
@@ -2532,8 +2655,8 @@
       <c r="G28" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H28" s="28" t="s">
-        <v>65</v>
+      <c r="H28" s="69" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="16.5" customHeight="1">
@@ -2541,7 +2664,7 @@
         <v>4</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C29" s="37" t="s">
         <v>11</v>
@@ -2554,8 +2677,8 @@
       <c r="G29" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H29" s="28" t="s">
-        <v>334</v>
+      <c r="H29" s="69" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1">
@@ -2576,8 +2699,8 @@
       <c r="G30" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H30" s="28" t="s">
-        <v>67</v>
+      <c r="H30" s="69" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="16.5" customHeight="1">
@@ -2588,7 +2711,7 @@
         <v>19</v>
       </c>
       <c r="C31" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>11</v>
@@ -2598,11 +2721,11 @@
       <c r="G31" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H31" s="28" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="16.5" customHeight="1">
+      <c r="H31" s="69" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="30.75" customHeight="1">
       <c r="A32" s="37">
         <v>6</v>
       </c>
@@ -2620,8 +2743,8 @@
       <c r="G32" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H32" s="28" t="s">
-        <v>68</v>
+      <c r="H32" s="69" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="16.5" customHeight="1">
@@ -2629,7 +2752,7 @@
         <v>7</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" s="37" t="s">
         <v>11</v>
@@ -2642,8 +2765,8 @@
       <c r="G33" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H33" s="28" t="s">
-        <v>70</v>
+      <c r="H33" s="69" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="16.5" customHeight="1">
@@ -2654,7 +2777,7 @@
         <v>39</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D34" s="37" t="s">
         <v>11</v>
@@ -2664,13 +2787,13 @@
       <c r="G34" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="H34" s="28" t="s">
-        <v>72</v>
+      <c r="H34" s="69" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="16.5" customHeight="1">
       <c r="A35" s="37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B35" s="37"/>
       <c r="C35" s="37"/>
@@ -2678,7 +2801,7 @@
       <c r="E35" s="41"/>
       <c r="F35" s="41"/>
       <c r="G35" s="37"/>
-      <c r="H35" s="28"/>
+      <c r="H35" s="69"/>
     </row>
     <row r="36" spans="1:8" ht="16.5" customHeight="1">
       <c r="A36" s="37">
@@ -2698,7 +2821,7 @@
       <c r="G36" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="H36" s="28"/>
+      <c r="H36" s="69"/>
     </row>
     <row r="37" spans="1:8" ht="16.5" customHeight="1">
       <c r="A37" s="37">
@@ -2718,25 +2841,25 @@
       <c r="G37" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="H37" s="28"/>
+      <c r="H37" s="69"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="54" t="s">
-        <v>75</v>
-      </c>
-      <c r="B38" s="55"/>
-      <c r="C38" s="55"/>
-      <c r="D38" s="56"/>
+      <c r="A38" s="56" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="57"/>
+      <c r="C38" s="57"/>
+      <c r="D38" s="58"/>
       <c r="E38" s="43">
-        <f>SUM(E27:E37)</f>
-        <v>0</v>
+        <f>SUM(E26:E37)</f>
+        <v>11000</v>
       </c>
       <c r="F38" s="43">
-        <f>SUM(F27:F37)</f>
-        <v>0</v>
+        <f>SUM(F26:F37)</f>
+        <v>11000</v>
       </c>
       <c r="G38" s="42"/>
-      <c r="H38" s="28"/>
+      <c r="H38" s="69"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:G19"/>
@@ -2749,7 +2872,7 @@
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2773,28 +2896,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1">
+      <c r="A3" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="59" t="s">
-        <v>77</v>
-      </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="56"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="26"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -2805,25 +2928,25 @@
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="16.5" customHeight="1">
@@ -2843,16 +2966,16 @@
         <v>11</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="I5" s="13" t="s">
         <v>87</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.5" customHeight="1">
@@ -2872,19 +2995,19 @@
         <v>11</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>90</v>
-      </c>
       <c r="H6" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="16.5" customHeight="1">
+    </row>
+    <row r="7" spans="1:9" ht="33" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>48</v>
       </c>
@@ -2901,16 +3024,16 @@
         <v>11</v>
       </c>
       <c r="F7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="12">
+        <v>46234</v>
+      </c>
+      <c r="H7" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>92</v>
-      </c>
       <c r="I7" s="13" t="s">
-        <v>88</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="26.25" customHeight="1">
@@ -2930,16 +3053,16 @@
         <v>11</v>
       </c>
       <c r="F8" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="14" t="s">
         <v>94</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.5" customHeight="1">
@@ -2954,16 +3077,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="56"/>
+      <c r="A10" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="58"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -2974,25 +3097,25 @@
         <v>3</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="G11" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="I11" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="31.5" customHeight="1">
@@ -3003,7 +3126,7 @@
         <v>20</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>11</v>
@@ -3015,13 +3138,13 @@
         <v>46106</v>
       </c>
       <c r="G12" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="13" t="s">
         <v>101</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="I12" s="13" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="16.5" customHeight="1">
@@ -3032,7 +3155,7 @@
         <v>46</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>11</v>
@@ -3045,10 +3168,10 @@
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="13" t="s">
         <v>87</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="16.5" customHeight="1">
@@ -3059,7 +3182,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>11</v>
@@ -3072,10 +3195,10 @@
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="13" t="s">
         <v>87</v>
-      </c>
-      <c r="I14" s="13" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30.75" customHeight="1">
@@ -3086,7 +3209,7 @@
         <v>54</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D15" s="8">
         <v>5</v>
@@ -3099,10 +3222,10 @@
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="16.5" customHeight="1">
@@ -3113,7 +3236,7 @@
         <v>51</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D16" s="8">
         <v>15</v>
@@ -3126,10 +3249,10 @@
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="16.5" customHeight="1">
@@ -3137,10 +3260,10 @@
         <v>39</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D17" s="8">
         <v>6</v>
@@ -3153,10 +3276,10 @@
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="16.5" customHeight="1">
@@ -3171,16 +3294,16 @@
       <c r="I18" s="13"/>
     </row>
     <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="59" t="s">
-        <v>111</v>
-      </c>
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="56"/>
+      <c r="A19" s="61" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="58"/>
       <c r="I19" s="26"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
@@ -3191,25 +3314,25 @@
         <v>3</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="16.5" customHeight="1">
@@ -3220,10 +3343,10 @@
         <v>27</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E21" s="8">
         <v>0</v>
@@ -3233,10 +3356,10 @@
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="16.5" customHeight="1">
@@ -3247,23 +3370,23 @@
         <v>14</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E22" s="8">
         <v>0</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="13" t="s">
         <v>87</v>
-      </c>
-      <c r="I22" s="13" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="30.75" customHeight="1">
@@ -3274,7 +3397,7 @@
         <v>17</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>11</v>
@@ -3287,10 +3410,10 @@
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="16.5" customHeight="1">
@@ -3305,16 +3428,16 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A25" s="59" t="s">
-        <v>119</v>
-      </c>
-      <c r="B25" s="55"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="56"/>
+      <c r="A25" s="61" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="57"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="57"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="58"/>
       <c r="I25" s="26"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
@@ -3325,25 +3448,25 @@
         <v>3</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="F26" s="4" t="s">
-        <v>123</v>
-      </c>
       <c r="G26" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="16.5" customHeight="1">
@@ -3351,51 +3474,53 @@
         <v>29</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="8">
         <v>480</v>
       </c>
       <c r="D27" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="F27" s="8" t="s">
         <v>125</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>126</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I27" s="13"/>
+      <c r="I27" s="14" t="s">
+        <v>342</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="33" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C28" s="8">
         <v>500</v>
       </c>
       <c r="D28" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>129</v>
-      </c>
       <c r="F28" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8" t="s">
         <v>11</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="33" customHeight="1">
@@ -3409,44 +3534,44 @@
         <v>900</v>
       </c>
       <c r="D29" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="F29" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="G29" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="H29" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="I29" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="H29" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="I29" s="14" t="s">
+    </row>
+    <row r="32" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A32" s="60" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A32" s="58" t="s">
-        <v>136</v>
-      </c>
-      <c r="B32" s="52"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
+      <c r="B32" s="54"/>
+      <c r="C32" s="54"/>
+      <c r="D32" s="54"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="54"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="54"/>
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1">
       <c r="A35" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="16.5">
@@ -3457,25 +3582,25 @@
         <v>3</v>
       </c>
       <c r="C37" s="49" t="s">
+        <v>77</v>
+      </c>
+      <c r="D37" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="49" t="s">
+      <c r="E37" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="E37" s="49" t="s">
+      <c r="F37" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="F37" s="49" t="s">
+      <c r="G37" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="G37" s="49" t="s">
+      <c r="H37" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="H37" s="49" t="s">
+      <c r="I37" s="49" t="s">
         <v>83</v>
-      </c>
-      <c r="I37" s="49" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="16.5">
@@ -3486,54 +3611,54 @@
         <v>59</v>
       </c>
       <c r="C38" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="D38" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="37" t="s">
+      <c r="G38" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="G38" s="37" t="s">
+      <c r="H38" s="44" t="s">
+        <v>86</v>
+      </c>
+      <c r="I38" s="68" t="s">
         <v>140</v>
-      </c>
-      <c r="H38" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="I38" s="45" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16.5">
       <c r="A39" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B39" s="37" t="s">
-        <v>62</v>
-      </c>
       <c r="C39" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="D39" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="D39" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="37" t="s">
+      <c r="G39" s="37" t="s">
         <v>143</v>
       </c>
-      <c r="G39" s="37" t="s">
+      <c r="H39" s="44" t="s">
+        <v>86</v>
+      </c>
+      <c r="I39" s="45" t="s">
         <v>144</v>
-      </c>
-      <c r="H39" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="I39" s="45" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16.5">
@@ -3541,31 +3666,31 @@
         <v>42</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C40" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="D40" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="37" t="s">
         <v>146</v>
       </c>
-      <c r="D40" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="37" t="s">
+      <c r="G40" s="37" t="s">
         <v>147</v>
       </c>
-      <c r="G40" s="37" t="s">
-        <v>148</v>
-      </c>
       <c r="H40" s="46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I40" s="45"/>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="16.5">
@@ -3576,36 +3701,36 @@
         <v>3</v>
       </c>
       <c r="C43" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="49" t="s">
         <v>97</v>
       </c>
-      <c r="D43" s="49" t="s">
+      <c r="E43" s="49" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="E43" s="49" t="s">
-        <v>80</v>
-      </c>
-      <c r="F43" s="49" t="s">
-        <v>99</v>
-      </c>
       <c r="G43" s="49" t="s">
         <v>11</v>
       </c>
       <c r="H43" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="I43" s="49" t="s">
         <v>83</v>
-      </c>
-      <c r="I43" s="49" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="16.5">
       <c r="A44" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44" s="37" t="s">
         <v>11</v>
       </c>
       <c r="C44" s="37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D44" s="37" t="s">
         <v>11</v>
@@ -3618,7 +3743,7 @@
       </c>
       <c r="G44" s="37"/>
       <c r="H44" s="44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I44" s="45"/>
     </row>
@@ -3630,7 +3755,7 @@
         <v>11</v>
       </c>
       <c r="C45" s="37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D45" s="37" t="s">
         <v>11</v>
@@ -3639,25 +3764,25 @@
         <v>11</v>
       </c>
       <c r="F45" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G45" s="37"/>
       <c r="H45" s="44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I45" s="45" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="16.5">
       <c r="A46" s="37" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B46" s="37" t="s">
-        <v>46</v>
-      </c>
-      <c r="C46" s="37" t="s">
-        <v>103</v>
+        <v>70</v>
+      </c>
+      <c r="C46" s="51" t="s">
+        <v>335</v>
       </c>
       <c r="D46" s="37" t="s">
         <v>11</v>
@@ -3668,82 +3793,86 @@
       <c r="F46" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="G46" s="37"/>
+      <c r="G46" s="37" t="s">
+        <v>11</v>
+      </c>
       <c r="H46" s="44" t="s">
-        <v>152</v>
-      </c>
-      <c r="I46" s="45" t="s">
+        <v>91</v>
+      </c>
+      <c r="I46" s="47" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="39" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="16.5">
-      <c r="A47" s="37" t="s">
-        <v>69</v>
-      </c>
-      <c r="B47" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="C47" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="D47" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F47" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="37"/>
-      <c r="H47" s="44" t="s">
-        <v>152</v>
-      </c>
-      <c r="I47" s="45"/>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" s="39" t="s">
+    <row r="49" spans="1:9" ht="16.5">
+      <c r="A49" s="49" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="49" t="s">
+        <v>3</v>
+      </c>
+      <c r="C49" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="G49" s="49" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="I49" s="49" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="16.5">
+      <c r="A50" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="C50" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="44" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="16.5">
-      <c r="A50" s="49" t="s">
-        <v>2</v>
-      </c>
-      <c r="B50" s="49" t="s">
-        <v>3</v>
-      </c>
-      <c r="C50" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="H50" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="I50" s="49" t="s">
-        <v>84</v>
-      </c>
+      <c r="I50" s="45"/>
     </row>
     <row r="51" spans="1:9" ht="16.5">
       <c r="A51" s="37" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="B51" s="37" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C51" s="37" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="D51" s="37" t="s">
         <v>11</v>
@@ -3754,23 +3883,23 @@
       <c r="F51" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="G51" s="37" t="s">
-        <v>11</v>
-      </c>
+      <c r="G51" s="37"/>
       <c r="H51" s="44" t="s">
-        <v>155</v>
-      </c>
-      <c r="I51" s="47"/>
+        <v>151</v>
+      </c>
+      <c r="I51" s="45" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="52" spans="1:9" ht="16.5">
       <c r="A52" s="37" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="B52" s="37" t="s">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="C52" s="37" t="s">
-        <v>11</v>
+        <v>104</v>
       </c>
       <c r="D52" s="37" t="s">
         <v>11</v>
@@ -3781,11 +3910,9 @@
       <c r="F52" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="G52" s="37" t="s">
-        <v>11</v>
-      </c>
+      <c r="G52" s="37"/>
       <c r="H52" s="44" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I52" s="45"/>
     </row>
@@ -3843,24 +3970,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A2" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="53" t="s">
-        <v>157</v>
-      </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -3873,13 +4000,13 @@
         <v>3</v>
       </c>
       <c r="D3" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" customHeight="1">
@@ -3896,7 +4023,7 @@
         <v>50000</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F4" s="8"/>
     </row>
@@ -3914,7 +4041,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F5" s="8"/>
     </row>
@@ -3932,7 +4059,7 @@
         <v>27000</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -3950,10 +4077,10 @@
         <v>20000</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
@@ -3964,13 +4091,13 @@
         <v>22</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D8" s="8">
         <v>60000</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F8" s="8"/>
     </row>
@@ -3988,15 +4115,15 @@
         <v>20000</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" customHeight="1">
       <c r="A10" s="8" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>48</v>
@@ -4008,7 +4135,7 @@
         <v>30000</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -4020,19 +4147,19 @@
         <v>29</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D11" s="8">
         <v>20000</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="16.5" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>41</v>
@@ -4044,7 +4171,7 @@
         <v>30000</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F12" s="8"/>
     </row>
@@ -4062,7 +4189,7 @@
         <v>19000</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F13" s="8"/>
     </row>
@@ -4080,10 +4207,10 @@
         <v>0</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" customHeight="1">
@@ -4094,13 +4221,13 @@
         <v>39</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D15" s="8">
         <v>50000</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -4118,7 +4245,7 @@
         <v>20000</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F16" s="8"/>
     </row>
@@ -4136,7 +4263,7 @@
         <v>71000</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F17" s="8"/>
     </row>
@@ -4154,10 +4281,10 @@
         <v>0</v>
       </c>
       <c r="E18" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>160</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="16.5" customHeight="1">
@@ -4174,23 +4301,23 @@
         <v>60000</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F19" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A21" s="53" t="s">
-        <v>162</v>
-      </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
+      <c r="A21" s="55" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
     </row>
     <row r="24" spans="1:6" ht="14.25">
       <c r="A24" s="38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15">
@@ -4204,18 +4331,18 @@
         <v>3</v>
       </c>
       <c r="D25" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="E25" s="40" t="s">
         <v>158</v>
       </c>
-      <c r="E25" s="40" t="s">
-        <v>159</v>
-      </c>
       <c r="F25" s="40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="33">
       <c r="A26" s="50" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="B26" s="37" t="s">
         <v>29</v>
@@ -4227,10 +4354,10 @@
         <v>11</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.5">
@@ -4238,59 +4365,59 @@
         <v>11</v>
       </c>
       <c r="B27" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="37" t="s">
-        <v>62</v>
-      </c>
       <c r="D27" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F27" s="37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="33">
       <c r="A28" s="50" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B28" s="37" t="s">
         <v>42</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D28" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16.5">
       <c r="A29" s="50" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B29" s="37" t="s">
         <v>19</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F29" s="50" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16.5">
@@ -4298,7 +4425,7 @@
         <v>11</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C30" s="37" t="s">
         <v>11</v>
@@ -4307,10 +4434,10 @@
         <v>11</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16.5">
@@ -4327,10 +4454,10 @@
         <v>11</v>
       </c>
       <c r="E31" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F31" s="37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16.5">
@@ -4347,10 +4474,10 @@
         <v>11</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F32" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="16.5">
@@ -4358,7 +4485,7 @@
         <v>11</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" s="37" t="s">
         <v>11</v>
@@ -4367,10 +4494,10 @@
         <v>11</v>
       </c>
       <c r="E33" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F33" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5">
@@ -4381,16 +4508,16 @@
         <v>39</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D34" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4427,53 +4554,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
+      <c r="A3" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="60" t="s">
-        <v>168</v>
-      </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
@@ -4481,7 +4608,7 @@
         <v>42</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C5" s="8">
         <v>3</v>
@@ -4493,13 +4620,13 @@
         <v>3</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
@@ -4507,7 +4634,7 @@
         <v>42</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C6" s="8">
         <v>5</v>
@@ -4519,13 +4646,13 @@
         <v>5</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>182</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" customHeight="1">
@@ -4533,7 +4660,7 @@
         <v>36</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C7" s="8">
         <v>6</v>
@@ -4545,13 +4672,13 @@
         <v>6</v>
       </c>
       <c r="F7" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>186</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" customHeight="1">
@@ -4559,7 +4686,7 @@
         <v>36</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C8" s="8">
         <v>2</v>
@@ -4571,13 +4698,13 @@
         <v>2</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G8" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>188</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="33" customHeight="1">
@@ -4585,7 +4712,7 @@
         <v>36</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C9" s="8">
         <v>4</v>
@@ -4597,13 +4724,13 @@
         <v>4</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="33" customHeight="1">
@@ -4611,7 +4738,7 @@
         <v>36</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C10" s="37">
         <v>6</v>
@@ -4623,13 +4750,13 @@
         <v>6</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G10" s="37" t="s">
+        <v>192</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>193</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16.5" customHeight="1">
@@ -4637,7 +4764,7 @@
         <v>50</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C11" s="8">
         <v>6</v>
@@ -4649,13 +4776,13 @@
         <v>6</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="33" customHeight="1">
@@ -4663,7 +4790,7 @@
         <v>50</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C12" s="8">
         <v>1</v>
@@ -4675,10 +4802,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>11</v>
@@ -4689,7 +4816,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C13" s="8">
         <v>4</v>
@@ -4701,13 +4828,13 @@
         <v>4</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G13" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>198</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.5" customHeight="1">
@@ -4715,7 +4842,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C14" s="8">
         <v>2</v>
@@ -4727,13 +4854,13 @@
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>202</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
@@ -4741,48 +4868,48 @@
         <v>33</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>204</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>205</v>
       </c>
       <c r="D15" s="8">
         <v>0</v>
       </c>
       <c r="E15" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="G15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="8" t="s">
+    </row>
+    <row r="16" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A16" s="63" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="57"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="G16" s="58"/>
+      <c r="H16" s="8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A17" s="64" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="61" t="s">
-        <v>181</v>
-      </c>
-      <c r="G16" s="56"/>
-      <c r="H16" s="8" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A17" s="62" t="s">
-        <v>208</v>
-      </c>
-      <c r="B17" s="56"/>
+      <c r="B17" s="58"/>
       <c r="C17">
         <f>SUM(C5:C15)</f>
         <v>39</v>
@@ -4795,48 +4922,48 @@
         <f>SUM(E5:E15)</f>
         <v>39</v>
       </c>
-      <c r="F17" s="62" t="s">
-        <v>209</v>
-      </c>
-      <c r="G17" s="56"/>
+      <c r="F17" s="64" t="s">
+        <v>208</v>
+      </c>
+      <c r="G17" s="58"/>
       <c r="H17" s="23"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
-      <c r="A18" s="52"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
+      <c r="A18" s="54"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1">
       <c r="A19" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>214</v>
-      </c>
       <c r="G20" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H20" s="1"/>
     </row>
@@ -4942,7 +5069,7 @@
     </row>
     <row r="33" spans="1:9" ht="14.25" customHeight="1">
       <c r="A33" s="31" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="15">
@@ -4953,25 +5080,25 @@
         <v>3</v>
       </c>
       <c r="C34" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="D34" s="40" t="s">
         <v>216</v>
       </c>
-      <c r="D34" s="40" t="s">
+      <c r="E34" s="40" t="s">
         <v>217</v>
       </c>
-      <c r="E34" s="40" t="s">
+      <c r="F34" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="G34" s="40" t="s">
         <v>218</v>
       </c>
-      <c r="F34" s="40" t="s">
-        <v>172</v>
-      </c>
-      <c r="G34" s="40" t="s">
+      <c r="H34" s="40" t="s">
         <v>219</v>
       </c>
-      <c r="H34" s="40" t="s">
-        <v>220</v>
-      </c>
       <c r="I34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="33">
@@ -4982,7 +5109,7 @@
         <v>59</v>
       </c>
       <c r="C35" s="37" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D35" s="37">
         <v>4</v>
@@ -4994,13 +5121,13 @@
         <v>4</v>
       </c>
       <c r="G35" s="37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H35" s="37" t="s">
+        <v>221</v>
+      </c>
+      <c r="I35" t="s">
         <v>222</v>
-      </c>
-      <c r="I35" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="33">
@@ -5011,36 +5138,36 @@
         <v>59</v>
       </c>
       <c r="C36" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="I36" t="s">
         <v>224</v>
-      </c>
-      <c r="D36" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="H36" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="16.5">
       <c r="A37" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="37" t="s">
-        <v>62</v>
-      </c>
       <c r="C37" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D37" s="37">
         <v>6</v>
@@ -5052,21 +5179,21 @@
         <v>6</v>
       </c>
       <c r="G37" s="37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H37" s="37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="16.5">
       <c r="A38" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="37" t="s">
-        <v>62</v>
-      </c>
       <c r="C38" s="37" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D38" s="37">
         <v>12</v>
@@ -5081,10 +5208,10 @@
         <v>11</v>
       </c>
       <c r="H38" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="I38" t="s">
         <v>228</v>
-      </c>
-      <c r="I38" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="33">
@@ -5092,10 +5219,10 @@
         <v>42</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C39" s="37" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D39" s="37">
         <v>2</v>
@@ -5107,10 +5234,10 @@
         <v>2</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="33">
@@ -5118,10 +5245,10 @@
         <v>42</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D40" s="37">
         <v>4</v>
@@ -5133,13 +5260,13 @@
         <v>4</v>
       </c>
       <c r="G40" s="37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="33">
@@ -5147,10 +5274,10 @@
         <v>42</v>
       </c>
       <c r="B41" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C41" s="37" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D41" s="37">
         <v>6</v>
@@ -5165,7 +5292,7 @@
         <v>11</v>
       </c>
       <c r="H41" s="37" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -5203,147 +5330,147 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>232</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
+      <c r="A3" s="62" t="s">
         <v>233</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="60" t="s">
-        <v>234</v>
-      </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="49.5" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>48</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>241</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>245</v>
-      </c>
       <c r="E6" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="33" customHeight="1">
       <c r="A7" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>248</v>
-      </c>
       <c r="E7" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="33" customHeight="1">
       <c r="A8" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="E8" s="8" t="s">
+    </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1">
+      <c r="A11" s="62" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="60" t="s">
-        <v>254</v>
-      </c>
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="54"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1">
@@ -5474,24 +5601,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>260</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1">
+      <c r="A3" s="62" t="s">
         <v>261</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="60" t="s">
-        <v>262</v>
-      </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -5501,16 +5628,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>264</v>
-      </c>
       <c r="F4" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" customHeight="1">
@@ -5518,19 +5645,19 @@
         <v>29</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" s="8">
         <v>480</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E5" s="8">
         <v>480</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" customHeight="1">
@@ -5538,19 +5665,19 @@
         <v>22</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="8">
         <v>500</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E6" s="8">
         <v>500</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" customHeight="1">
@@ -5564,31 +5691,31 @@
         <v>900</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E7" s="8">
         <v>900</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="56"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="37">
         <v>500</v>
       </c>
       <c r="D8" s="37" t="s">
+        <v>265</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="37" t="s">
         <v>266</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="37" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" customHeight="1">
@@ -5602,28 +5729,28 @@
         <v>1800</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E9" s="37" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="63"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="56"/>
+      <c r="A10" s="65"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="58"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="62" t="s">
-        <v>208</v>
-      </c>
-      <c r="B11" s="56"/>
+      <c r="A11" s="64" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" s="58"/>
       <c r="C11" s="36">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -5638,18 +5765,18 @@
     <row r="12" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="13" spans="1:6" ht="16.5" customHeight="1">
       <c r="A13" s="35" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>271</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>272</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>11</v>
@@ -5663,10 +5790,10 @@
     </row>
     <row r="15" spans="1:6" ht="16.5" customHeight="1">
       <c r="A15" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>273</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>274</v>
       </c>
       <c r="C15" s="8">
         <v>0</v>
@@ -5674,7 +5801,7 @@
     </row>
     <row r="16" spans="1:6" ht="16.5" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>11</v>
@@ -5684,21 +5811,21 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="61" t="s">
-        <v>276</v>
-      </c>
-      <c r="B17" s="55"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="56"/>
+      <c r="A17" s="63" t="s">
+        <v>275</v>
+      </c>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="58"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C18" s="11">
         <v>0</v>
@@ -5710,15 +5837,15 @@
     <row r="19" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="20" spans="1:6" ht="16.5" customHeight="1">
       <c r="A20" s="35" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16.5" customHeight="1">
       <c r="A21" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>278</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>279</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>11</v>
@@ -5735,38 +5862,38 @@
     </row>
     <row r="22" spans="1:6" ht="16.5" customHeight="1">
       <c r="A22" s="24" t="s">
+        <v>279</v>
+      </c>
+      <c r="B22" s="25" t="s">
         <v>280</v>
       </c>
-      <c r="B22" s="25" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="61" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="56"/>
+      <c r="A23" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" s="57"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="58"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
       <c r="A26" s="33" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.25" customHeight="1">
       <c r="A29" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15">
@@ -5777,16 +5904,16 @@
         <v>3</v>
       </c>
       <c r="C30" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="D30" s="48" t="s">
+        <v>255</v>
+      </c>
+      <c r="E30" s="48" t="s">
         <v>263</v>
       </c>
-      <c r="D30" s="48" t="s">
-        <v>256</v>
-      </c>
-      <c r="E30" s="48" t="s">
-        <v>264</v>
-      </c>
       <c r="F30" s="48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16.5">
@@ -5800,33 +5927,33 @@
         <v>980</v>
       </c>
       <c r="D31" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E31" s="37" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="37" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16.5">
       <c r="A32" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="37" t="s">
         <v>61</v>
-      </c>
-      <c r="B32" s="37" t="s">
-        <v>62</v>
       </c>
       <c r="C32" s="37">
         <v>500</v>
       </c>
       <c r="D32" s="37" t="s">
+        <v>285</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="37" t="s">
         <v>286</v>
-      </c>
-      <c r="E32" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="37" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="16.5">
@@ -5834,24 +5961,24 @@
         <v>42</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C33" s="37">
         <v>580</v>
       </c>
       <c r="D33" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E33" s="37" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="37" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5">
       <c r="A34" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B34" s="34" t="s">
         <v>11</v>
@@ -5860,13 +5987,13 @@
         <v>11</v>
       </c>
       <c r="D34" s="37" t="s">
+        <v>288</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="37" t="s">
         <v>289</v>
-      </c>
-      <c r="E34" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="37" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="16.5">
@@ -5880,13 +6007,13 @@
         <v>11</v>
       </c>
       <c r="D35" s="37" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E35" s="37" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -5921,28 +6048,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="53" t="s">
+        <v>291</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="55" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="53" t="s">
-        <v>293</v>
-      </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -5952,22 +6079,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
@@ -5978,7 +6105,7 @@
         <v>43</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>11</v>
@@ -5990,7 +6117,7 @@
         <v>11</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>11</v>
@@ -6004,7 +6131,7 @@
         <v>37</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
@@ -6016,7 +6143,7 @@
         <v>11</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>11</v>
@@ -6030,7 +6157,7 @@
         <v>49</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>11</v>
@@ -6042,7 +6169,7 @@
         <v>11</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>11</v>
@@ -6056,7 +6183,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>11</v>
@@ -6068,7 +6195,7 @@
         <v>11</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>11</v>
@@ -6082,19 +6209,19 @@
         <v>20</v>
       </c>
       <c r="C8" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>300</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>11</v>
@@ -6108,19 +6235,19 @@
         <v>46</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>300</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>11</v>
@@ -6134,7 +6261,7 @@
         <v>54</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>11</v>
@@ -6146,7 +6273,7 @@
         <v>11</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>11</v>
@@ -6154,7 +6281,7 @@
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1">
       <c r="A13" s="31" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15">
@@ -6165,22 +6292,22 @@
         <v>3</v>
       </c>
       <c r="C14" s="40" t="s">
+        <v>293</v>
+      </c>
+      <c r="D14" s="40" t="s">
         <v>294</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="E14" s="40" t="s">
         <v>295</v>
       </c>
-      <c r="E14" s="40" t="s">
+      <c r="F14" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="40" t="s">
         <v>296</v>
       </c>
-      <c r="F14" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" s="40" t="s">
+      <c r="H14" s="40" t="s">
         <v>297</v>
-      </c>
-      <c r="H14" s="40" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5">
@@ -6191,19 +6318,19 @@
         <v>59</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D15" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F15" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H15" s="37" t="s">
         <v>11</v>
@@ -6211,25 +6338,25 @@
     </row>
     <row r="16" spans="1:8" ht="16.5">
       <c r="A16" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="37" t="s">
-        <v>62</v>
-      </c>
       <c r="C16" s="37" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D16" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F16" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H16" s="37" t="s">
         <v>11</v>
@@ -6240,22 +6367,22 @@
         <v>42</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D17" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F17" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G17" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H17" s="37" t="s">
         <v>11</v>
@@ -6263,13 +6390,13 @@
     </row>
     <row r="18" spans="1:8" ht="16.5">
       <c r="A18" s="37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B18" s="37" t="s">
         <v>54</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D18" s="37" t="s">
         <v>11</v>
@@ -6281,10 +6408,10 @@
         <v>11</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -6307,7 +6434,7 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="14" style="32" customWidth="1"/>
@@ -6319,90 +6446,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
-        <v>306</v>
-      </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
+      <c r="A1" s="67" t="s">
+        <v>305</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>309</v>
-      </c>
       <c r="F2" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="21.95" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>50</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="19" t="s">
         <v>312</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="F3" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D4" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>316</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>313</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="21.95" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>11</v>
@@ -6416,36 +6543,36 @@
         <v>26</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="21" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>320</v>
-      </c>
       <c r="F6" s="10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="21.95" customHeight="1">
+    <row r="7" spans="1:6" ht="43.5" customHeight="1">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="70" t="s">
+        <v>318</v>
+      </c>
+      <c r="D7" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="71" t="s">
         <v>319</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>11</v>
+      <c r="F7" s="72" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21.95" customHeight="1">
@@ -6453,16 +6580,16 @@
         <v>11</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="E8" s="20" t="s">
         <v>321</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>322</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>323</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>11</v>
@@ -6476,13 +6603,13 @@
         <v>19</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>11</v>
@@ -6490,19 +6617,19 @@
     </row>
     <row r="10" spans="1:6" ht="21.95" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>11</v>
+        <v>323</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>11</v>
@@ -6510,19 +6637,19 @@
     </row>
     <row r="11" spans="1:6" ht="21.95" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>327</v>
+        <v>11</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>328</v>
-      </c>
-      <c r="E11" s="20" t="s">
         <v>325</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>165</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>11</v>
@@ -6533,38 +6660,18 @@
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A13" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>311</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>166</v>
-      </c>
-      <c r="F13" s="10" t="s">
         <v>11</v>
       </c>
     </row>
@@ -6573,7 +6680,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="E3:E13">
+  <conditionalFormatting sqref="E3:E12">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"✅*"</formula>
     </cfRule>

</xml_diff>